<commit_message>
chore(templates): regenerate SAP templates with original headers from Control Daily Repair by SAP.xlsx
</commit_message>
<xml_diff>
--- a/public/template-monitoring-mp-repair.xlsx
+++ b/public/template-monitoring-mp-repair.xlsx
@@ -32,8 +32,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="9">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="58" formatCode="m/d/yy"/>
+    <numFmt numFmtId="176" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_-&quot;Rp&quot;* #,##0.00_-;\-&quot;Rp&quot;* #,##0.00_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="178" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="179" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="180" formatCode="0.000"/>
+    <numFmt numFmtId="181" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="182" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -397,7 +405,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:E2"/>
+  <cols>
+    <col min="1" max="1" customWidth="1" width="3.85714285714286"/>
+    <col min="2" max="2" customWidth="1" width="10.8571428571429"/>
+    <col min="3" max="3" customWidth="1" width="15.7142857142857"/>
+    <col min="4" max="4" customWidth="1" width="5.28571428571429"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,73 +429,11 @@
       <c r="E1" t="str">
         <v>Gudang</v>
       </c>
-      <c r="F1" t="str">
-        <v>Kepala Regu</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2026-09-18</v>
-      </c>
-      <c r="C2">
-        <v>5</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Shift 1</v>
-      </c>
-      <c r="E2" t="str">
-        <v>1</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Budi</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2026-09-18</v>
-      </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Shift 2</v>
-      </c>
-      <c r="E3" t="str">
-        <v>5</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Suharto</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2026-09-18</v>
-      </c>
-      <c r="C4">
-        <v>6</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Shift 1</v>
-      </c>
-      <c r="E4" t="str">
-        <v>13</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Hadad</v>
-      </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>